<commit_message>
swarm ex weekly updates
</commit_message>
<xml_diff>
--- a/SWARM-EX/Planning/Personal Waterfall Chart Justin Le.xlsx
+++ b/SWARM-EX/Planning/Personal Waterfall Chart Justin Le.xlsx
@@ -2376,7 +2376,7 @@
       </c>
       <c r="E3" s="22" t="n">
         <f aca="false">SUM(F3:W3)</f>
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F3" s="23" t="n">
         <f aca="false">F4+F7+F11+F14</f>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="I3" s="23" t="n">
         <f aca="false">I4+I7+I11+I14</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J3" s="23" t="n">
         <f aca="false">J4+J7+J11+J14</f>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="E4" s="32" t="n">
         <f aca="false">SUM(F4:W4)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F4" s="33" t="n">
         <f aca="false">SUM(F5:F6)</f>
@@ -2485,7 +2485,7 @@
       </c>
       <c r="I4" s="33" t="n">
         <f aca="false">SUM(I5:I6)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J4" s="33" t="n">
         <f aca="false">SUM(J5:J6)</f>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="E5" s="32" t="n">
         <f aca="false">SUM(F5:W5)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" s="42" t="n">
         <v>1</v>
@@ -2579,7 +2579,9 @@
       <c r="H5" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="I5" s="33"/>
+      <c r="I5" s="33" t="n">
+        <v>1</v>
+      </c>
       <c r="J5" s="33"/>
       <c r="K5" s="33"/>
       <c r="L5" s="33"/>
@@ -2619,7 +2621,7 @@
       </c>
       <c r="E6" s="50" t="n">
         <f aca="false">SUM(F6:W6)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F6" s="51" t="n">
         <v>2</v>
@@ -2630,7 +2632,9 @@
       <c r="H6" s="52" t="n">
         <v>2</v>
       </c>
-      <c r="I6" s="52"/>
+      <c r="I6" s="52" t="n">
+        <v>2</v>
+      </c>
       <c r="J6" s="52"/>
       <c r="K6" s="52"/>
       <c r="L6" s="52"/>
@@ -2669,7 +2673,7 @@
       </c>
       <c r="E7" s="32" t="n">
         <f aca="false">SUM(F7:W7)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F7" s="56" t="n">
         <f aca="false">SUM(F8:F10)</f>
@@ -2685,7 +2689,7 @@
       </c>
       <c r="I7" s="56" t="n">
         <f aca="false">SUM(I8:I10)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J7" s="56" t="n">
         <f aca="false">SUM(J8:J10)</f>
@@ -2766,7 +2770,7 @@
       </c>
       <c r="E8" s="32" t="n">
         <f aca="false">SUM(F8:W8)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8" s="42" t="n">
         <v>1</v>
@@ -2777,7 +2781,9 @@
       <c r="H8" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="33"/>
+      <c r="I8" s="33" t="n">
+        <v>1</v>
+      </c>
       <c r="J8" s="33"/>
       <c r="K8" s="33"/>
       <c r="L8" s="33"/>
@@ -2815,7 +2821,7 @@
       </c>
       <c r="E9" s="32" t="n">
         <f aca="false">SUM(F9:W9)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" s="42" t="n">
         <v>1</v>
@@ -2826,7 +2832,9 @@
       <c r="H9" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="33"/>
+      <c r="I9" s="33" t="n">
+        <v>1</v>
+      </c>
       <c r="J9" s="33"/>
       <c r="K9" s="33"/>
       <c r="L9" s="33"/>
@@ -2860,7 +2868,7 @@
       </c>
       <c r="E10" s="50" t="n">
         <f aca="false">SUM(F10:W10)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F10" s="51" t="n">
         <v>2</v>
@@ -2871,7 +2879,9 @@
       <c r="H10" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="I10" s="52"/>
+      <c r="I10" s="52" t="n">
+        <v>1</v>
+      </c>
       <c r="J10" s="52"/>
       <c r="K10" s="52"/>
       <c r="L10" s="52"/>
@@ -2906,7 +2916,7 @@
       </c>
       <c r="E11" s="32" t="n">
         <f aca="false">SUM(F11:W11)</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F11" s="56" t="n">
         <f aca="false">SUM(F12:F13)</f>
@@ -2922,7 +2932,7 @@
       </c>
       <c r="I11" s="56" t="n">
         <f aca="false">SUM(I12:I13)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J11" s="56" t="n">
         <f aca="false">SUM(J12:J13)</f>
@@ -3048,7 +3058,7 @@
       </c>
       <c r="E13" s="50" t="n">
         <f aca="false">SUM(F13:W13)</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F13" s="51" t="n">
         <v>4</v>
@@ -3059,7 +3069,9 @@
       <c r="H13" s="52" t="n">
         <v>4</v>
       </c>
-      <c r="I13" s="52"/>
+      <c r="I13" s="52" t="n">
+        <v>2</v>
+      </c>
       <c r="J13" s="52"/>
       <c r="K13" s="52"/>
       <c r="L13" s="52"/>
@@ -3285,7 +3297,7 @@
       </c>
       <c r="E17" s="22" t="n">
         <f aca="false">SUM(F17:W17)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F17" s="68" t="n">
         <f aca="false">F18+F21+F23+F26</f>
@@ -3301,7 +3313,7 @@
       </c>
       <c r="I17" s="68" t="n">
         <f aca="false">I18+I21+I23+I26</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17" s="68" t="n">
         <f aca="false">J18+J21+J23+J26</f>
@@ -3556,7 +3568,7 @@
       </c>
       <c r="E21" s="32" t="n">
         <f aca="false">SUM(F21:W21)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21" s="56" t="n">
         <f aca="false">SUM(F22)</f>
@@ -3572,7 +3584,7 @@
       </c>
       <c r="I21" s="56" t="n">
         <f aca="false">SUM(I22)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" s="56" t="n">
         <f aca="false">SUM(J22)</f>
@@ -3651,14 +3663,16 @@
       </c>
       <c r="E22" s="32" t="n">
         <f aca="false">SUM(F22:W22)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" s="42"/>
       <c r="G22" s="33"/>
       <c r="H22" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="I22" s="33"/>
+      <c r="I22" s="33" t="n">
+        <v>1</v>
+      </c>
       <c r="J22" s="33"/>
       <c r="K22" s="33"/>
       <c r="L22" s="33"/>
@@ -3974,7 +3988,7 @@
       </c>
       <c r="E29" s="22" t="n">
         <f aca="false">SUM(F29:W29)</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F29" s="68" t="n">
         <f aca="false">F30+F41+F47</f>
@@ -3990,7 +4004,7 @@
       </c>
       <c r="I29" s="68" t="n">
         <f aca="false">I30+I41+I47</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J29" s="68" t="n">
         <f aca="false">J30+J41+J47</f>
@@ -4063,7 +4077,7 @@
       </c>
       <c r="E30" s="32" t="n">
         <f aca="false">SUM(F30:W30)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F30" s="56" t="n">
         <f aca="false">SUM(F31:F40)</f>
@@ -4079,7 +4093,7 @@
       </c>
       <c r="I30" s="34" t="n">
         <f aca="false">SUM(I31:I40)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J30" s="34" t="n">
         <f aca="false">SUM(J31:J40)</f>
@@ -4156,14 +4170,16 @@
       </c>
       <c r="E31" s="32" t="n">
         <f aca="false">SUM(F31:W31)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F31" s="42"/>
       <c r="G31" s="33"/>
       <c r="H31" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="I31" s="77"/>
+      <c r="I31" s="77" t="n">
+        <v>1</v>
+      </c>
       <c r="J31" s="33"/>
       <c r="K31" s="33"/>
       <c r="L31" s="33"/>
@@ -4197,12 +4213,14 @@
       </c>
       <c r="E32" s="32" t="n">
         <f aca="false">SUM(F32:W32)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32" s="42"/>
       <c r="G32" s="33"/>
       <c r="H32" s="33"/>
-      <c r="I32" s="77"/>
+      <c r="I32" s="77" t="n">
+        <v>1</v>
+      </c>
       <c r="J32" s="33"/>
       <c r="K32" s="33"/>
       <c r="L32" s="33"/>
@@ -4549,7 +4567,7 @@
       </c>
       <c r="E41" s="32" t="n">
         <f aca="false">SUM(F41:W41)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F41" s="56" t="n">
         <f aca="false">SUM(F42:F46)</f>
@@ -4565,7 +4583,7 @@
       </c>
       <c r="I41" s="34" t="n">
         <f aca="false">SUM(I42:I46)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J41" s="34" t="n">
         <f aca="false">SUM(J42:J46)</f>
@@ -4642,12 +4660,14 @@
       </c>
       <c r="E42" s="32" t="n">
         <f aca="false">SUM(F42:W42)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F42" s="42"/>
       <c r="G42" s="33"/>
       <c r="H42" s="33"/>
-      <c r="I42" s="33"/>
+      <c r="I42" s="33" t="n">
+        <v>2</v>
+      </c>
       <c r="J42" s="33"/>
       <c r="K42" s="33"/>
       <c r="L42" s="33"/>
@@ -4681,12 +4701,14 @@
       </c>
       <c r="E43" s="32" t="n">
         <f aca="false">SUM(F43:W43)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F43" s="42"/>
       <c r="G43" s="33"/>
       <c r="H43" s="33"/>
-      <c r="I43" s="33"/>
+      <c r="I43" s="33" t="n">
+        <v>1</v>
+      </c>
       <c r="J43" s="33"/>
       <c r="K43" s="33"/>
       <c r="L43" s="33"/>
@@ -5245,7 +5267,7 @@
       </c>
       <c r="E56" s="82" t="n">
         <f aca="false">E29+E17+E3</f>
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="F56" s="82" t="n">
         <f aca="false">F29+F17+F3</f>
@@ -5261,7 +5283,7 @@
       </c>
       <c r="I56" s="82" t="n">
         <f aca="false">I29+I17+I3</f>
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="J56" s="82" t="n">
         <f aca="false">J29+J17+J3</f>
@@ -5400,7 +5422,7 @@
       </c>
       <c r="E58" s="84" t="n">
         <f aca="false">E57-E56</f>
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="F58" s="84" t="n">
         <f aca="false">F57-F56</f>
@@ -5416,7 +5438,7 @@
       </c>
       <c r="I58" s="84" t="n">
         <f aca="false">I57-I56</f>
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="J58" s="84" t="n">
         <f aca="false">J57-J56</f>

</xml_diff>